<commit_message>
Actualización automática de base de datos
</commit_message>
<xml_diff>
--- a/LMI Base.xlsx
+++ b/LMI Base.xlsx
@@ -8,78 +8,79 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\alex1\Downloads\LMI\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7490922F-E1CC-473F-8F29-F6118EB781DB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D61601FE-001E-4874-AA52-8337C6468984}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Registro Liga" sheetId="1" r:id="rId1"/>
-    <sheet name="ChampionsLeague" sheetId="2" r:id="rId2"/>
-    <sheet name="CopaEstelar" sheetId="3" r:id="rId3"/>
-    <sheet name="Registro Champions" sheetId="4" r:id="rId4"/>
-    <sheet name="RegistroEstelar" sheetId="5" r:id="rId5"/>
-    <sheet name="BD" sheetId="6" r:id="rId6"/>
-    <sheet name="Lista" sheetId="7" r:id="rId7"/>
-    <sheet name="Clubes" sheetId="8" r:id="rId8"/>
-    <sheet name="Mercado" sheetId="9" r:id="rId9"/>
-    <sheet name="Campeones" sheetId="10" r:id="rId10"/>
-    <sheet name="RESPALDO" sheetId="11" r:id="rId11"/>
+    <sheet name="Renovaciones" sheetId="12" r:id="rId2"/>
+    <sheet name="ChampionsLeague" sheetId="2" r:id="rId3"/>
+    <sheet name="CopaEstelar" sheetId="3" r:id="rId4"/>
+    <sheet name="Registro Champions" sheetId="4" r:id="rId5"/>
+    <sheet name="RegistroEstelar" sheetId="5" r:id="rId6"/>
+    <sheet name="BD" sheetId="6" r:id="rId7"/>
+    <sheet name="Lista" sheetId="7" r:id="rId8"/>
+    <sheet name="Clubes" sheetId="8" r:id="rId9"/>
+    <sheet name="Mercado" sheetId="9" r:id="rId10"/>
+    <sheet name="Campeones" sheetId="10" r:id="rId11"/>
+    <sheet name="RESPALDO" sheetId="11" r:id="rId12"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">Clubes!$A$1:$H$19</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">Mercado!$A$1:$G$51</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Registro Champions'!$A$1:$D$122</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">Clubes!$A$1:$H$19</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">Mercado!$A$1:$G$51</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Registro Champions'!$A$1:$D$122</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Registro Liga'!$A$1:$D$251</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">RegistroEstelar!$A$1:$D$80</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">RegistroEstelar!$A$1:$D$80</definedName>
     <definedName name="AC_Milan">BD!$D$2:$D$24</definedName>
     <definedName name="AC_Milán">Lista!$E$2:$E$1048576</definedName>
     <definedName name="AcMilan">Lista!$E$2:$E$1048576</definedName>
-    <definedName name="Arsenal" localSheetId="5">BD!$J$2:$J$24</definedName>
+    <definedName name="Arsenal" localSheetId="6">BD!$J$2:$J$24</definedName>
     <definedName name="Arsenal">Lista!$K$2:$K$1048576</definedName>
     <definedName name="AstonVilla">Lista!$I$2:$I$1048576</definedName>
     <definedName name="Bayer_Munich">Lista!$O$2:$O$1048576</definedName>
-    <definedName name="Bayern_Leverkusen" localSheetId="5">BD!$E$2:$E$24</definedName>
+    <definedName name="Bayern_Leverkusen" localSheetId="6">BD!$E$2:$E$24</definedName>
     <definedName name="Bayern_Leverkusen">Lista!$F$2:$F$1048576</definedName>
     <definedName name="Bayern_Munich">BD!$N$2:$N$24</definedName>
-    <definedName name="Boca_Juniors" localSheetId="5">BD!$G$2:$G$24</definedName>
+    <definedName name="Boca_Juniors" localSheetId="6">BD!$G$2:$G$24</definedName>
     <definedName name="Boca_Juniors">Lista!$H$2:$H$1048576</definedName>
     <definedName name="BocaJuniors">Lista!$H$2:$H$1048576</definedName>
-    <definedName name="Como_1907" localSheetId="5">BD!$K$2:$K$24</definedName>
+    <definedName name="Como_1907" localSheetId="6">BD!$K$2:$K$24</definedName>
     <definedName name="COMO_1907">Lista!$L$2:$L$1048576</definedName>
     <definedName name="Como1907">Lista!$M$2:$M$1048576</definedName>
-    <definedName name="FC_Barcelona" localSheetId="5">BD!$C$2:$C$24</definedName>
+    <definedName name="FC_Barcelona" localSheetId="6">BD!$C$2:$C$24</definedName>
     <definedName name="FC_Barcelona">Lista!$C$2:$C$1048576</definedName>
     <definedName name="FcBarcelona">Lista!$C$2:$C$1048576</definedName>
-    <definedName name="Galatasaray" localSheetId="5">BD!$H$2:$H$24</definedName>
+    <definedName name="Galatasaray" localSheetId="6">BD!$H$2:$H$24</definedName>
     <definedName name="GALATASARAY">Lista!$I$2:$I$1048576</definedName>
-    <definedName name="Hellas_Verona" localSheetId="5">BD!$M$2:$M$24</definedName>
+    <definedName name="Hellas_Verona" localSheetId="6">BD!$M$2:$M$24</definedName>
     <definedName name="Hellas_Verona">Lista!$N$2:$N$1048576</definedName>
-    <definedName name="Inter_de_Milan" localSheetId="5">BD!$A$2:$A$24</definedName>
+    <definedName name="Inter_de_Milan" localSheetId="6">BD!$A$2:$A$24</definedName>
     <definedName name="Inter_de_Milan">Lista!$A$2:$A$1048576</definedName>
     <definedName name="InterMilan">Lista!$A$2:$A$1048576</definedName>
     <definedName name="Leverkusen">Lista!$F$2:$F$1048576</definedName>
-    <definedName name="Manchester_United" localSheetId="5">BD!$O$2:$O$24</definedName>
+    <definedName name="Manchester_United" localSheetId="6">BD!$O$2:$O$24</definedName>
     <definedName name="Manchester_United">Lista!$P$2:$P$1048576</definedName>
-    <definedName name="Melbourne_City" localSheetId="5">BD!#REF!</definedName>
+    <definedName name="Melbourne_City" localSheetId="6">BD!#REF!</definedName>
     <definedName name="Melbourne_City">Lista!$Q$2:$Q$1048576</definedName>
     <definedName name="PARIS_SAINT___GERMAIN">Lista!$J$2:$J$1048576</definedName>
-    <definedName name="PSG" localSheetId="5">BD!$I$2:$I$23</definedName>
+    <definedName name="PSG" localSheetId="6">BD!$I$2:$I$23</definedName>
     <definedName name="PSG">Lista!$K$2:$K$1048576</definedName>
-    <definedName name="RB_Leipzig" localSheetId="5">BD!$F$2:$F$24</definedName>
+    <definedName name="RB_Leipzig" localSheetId="6">BD!$F$2:$F$24</definedName>
     <definedName name="RB_LEIPZIG">Lista!$G$2:$G$1048576</definedName>
     <definedName name="RBLeipzig">Lista!$G$2:$G$1048576</definedName>
-    <definedName name="Real_Madrid" localSheetId="5">BD!$B$2:$B$24</definedName>
+    <definedName name="Real_Madrid" localSheetId="6">BD!$B$2:$B$24</definedName>
     <definedName name="Real_Madrid">Lista!$B$2:$B$1048576</definedName>
     <definedName name="RealMadrid">Lista!$B$2:$B$1048576</definedName>
     <definedName name="Sparta">Lista!$P$2:$P$1048576</definedName>
-    <definedName name="Terengganu_FC" localSheetId="5">BD!#REF!</definedName>
+    <definedName name="Terengganu_FC" localSheetId="6">BD!#REF!</definedName>
     <definedName name="Terengganu_FC">Lista!$D$2:$D$1048576</definedName>
     <definedName name="Terrengganu">Lista!$D$2:$D$1048576</definedName>
     <definedName name="Tottenham">Lista!$O$2:$O$1048576</definedName>
-    <definedName name="Tottenham_Hotspur" localSheetId="5">BD!$L$2:$L$24</definedName>
+    <definedName name="Tottenham_Hotspur" localSheetId="6">BD!$L$2:$L$24</definedName>
     <definedName name="Tottenham_Hotspur">Lista!$M$2:$M$1048576</definedName>
     <definedName name="United">Lista!$N$2:$N$1048576</definedName>
-    <definedName name="Wrexham" localSheetId="5">BD!$P$2:$P$24</definedName>
+    <definedName name="Wrexham" localSheetId="6">BD!$P$2:$P$24</definedName>
     <definedName name="WREXHAM">Lista!$R$2:$R$1048576</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
@@ -100,7 +101,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2475" uniqueCount="1080">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2555" uniqueCount="1084">
   <si>
     <t>Equipo</t>
   </si>
@@ -3340,6 +3341,18 @@
   </si>
   <si>
     <t>Eder Militao</t>
+  </si>
+  <si>
+    <t>Valor</t>
+  </si>
+  <si>
+    <t>Epico</t>
+  </si>
+  <si>
+    <t>Big Time</t>
+  </si>
+  <si>
+    <t>CT Fabio Cannavaro</t>
   </si>
 </sst>
 </file>
@@ -3416,7 +3429,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -3445,6 +3458,9 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -7122,6 +7138,314 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
+  <dimension ref="A1:G13"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="16.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.21875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15.6640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="16.44140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="5.77734375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="30.77734375" customWidth="1"/>
+    <col min="8" max="10" width="8.77734375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1" t="s">
+        <v>997</v>
+      </c>
+      <c r="C1" t="s">
+        <v>998</v>
+      </c>
+      <c r="D1" t="s">
+        <v>999</v>
+      </c>
+      <c r="E1" t="s">
+        <v>1000</v>
+      </c>
+      <c r="F1" t="s">
+        <v>1001</v>
+      </c>
+      <c r="G1" t="s">
+        <v>1002</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>464</v>
+      </c>
+      <c r="B2" t="s">
+        <v>1003</v>
+      </c>
+      <c r="C2" t="s">
+        <v>229</v>
+      </c>
+      <c r="D2" t="s">
+        <v>1004</v>
+      </c>
+      <c r="F2">
+        <v>1</v>
+      </c>
+      <c r="G2" t="s">
+        <v>1005</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>1006</v>
+      </c>
+      <c r="B3" t="s">
+        <v>1003</v>
+      </c>
+      <c r="C3" t="s">
+        <v>1004</v>
+      </c>
+      <c r="D3" t="s">
+        <v>229</v>
+      </c>
+      <c r="F3">
+        <v>1</v>
+      </c>
+      <c r="G3" t="s">
+        <v>1005</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>57</v>
+      </c>
+      <c r="B4" t="s">
+        <v>1003</v>
+      </c>
+      <c r="C4" t="s">
+        <v>234</v>
+      </c>
+      <c r="D4" t="s">
+        <v>55</v>
+      </c>
+      <c r="F4">
+        <v>1</v>
+      </c>
+      <c r="G4" t="s">
+        <v>1005</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>66</v>
+      </c>
+      <c r="B5" t="s">
+        <v>1003</v>
+      </c>
+      <c r="C5" t="s">
+        <v>55</v>
+      </c>
+      <c r="D5" t="s">
+        <v>234</v>
+      </c>
+      <c r="F5">
+        <v>1</v>
+      </c>
+      <c r="G5" t="s">
+        <v>1005</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>1007</v>
+      </c>
+      <c r="B6" t="s">
+        <v>1003</v>
+      </c>
+      <c r="C6" t="s">
+        <v>501</v>
+      </c>
+      <c r="D6" t="s">
+        <v>234</v>
+      </c>
+      <c r="E6">
+        <v>40</v>
+      </c>
+      <c r="F6">
+        <v>2</v>
+      </c>
+      <c r="G6" t="s">
+        <v>1005</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>267</v>
+      </c>
+      <c r="B7" t="s">
+        <v>1003</v>
+      </c>
+      <c r="C7" t="s">
+        <v>501</v>
+      </c>
+      <c r="D7" t="s">
+        <v>234</v>
+      </c>
+      <c r="E7">
+        <v>15</v>
+      </c>
+      <c r="F7">
+        <v>2</v>
+      </c>
+      <c r="G7" t="s">
+        <v>1005</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>1008</v>
+      </c>
+      <c r="B8" t="s">
+        <v>1003</v>
+      </c>
+      <c r="C8" t="s">
+        <v>234</v>
+      </c>
+      <c r="D8" t="s">
+        <v>497</v>
+      </c>
+      <c r="E8">
+        <v>0</v>
+      </c>
+      <c r="F8">
+        <v>2</v>
+      </c>
+      <c r="G8" t="s">
+        <v>1009</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>1010</v>
+      </c>
+      <c r="B9" t="s">
+        <v>1003</v>
+      </c>
+      <c r="C9" t="s">
+        <v>229</v>
+      </c>
+      <c r="D9" t="s">
+        <v>233</v>
+      </c>
+      <c r="E9">
+        <v>0</v>
+      </c>
+      <c r="F9">
+        <v>2</v>
+      </c>
+      <c r="G9" t="s">
+        <v>1009</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>1011</v>
+      </c>
+      <c r="B10" t="s">
+        <v>1003</v>
+      </c>
+      <c r="C10" t="s">
+        <v>233</v>
+      </c>
+      <c r="D10" t="s">
+        <v>229</v>
+      </c>
+      <c r="E10">
+        <v>0</v>
+      </c>
+      <c r="F10">
+        <v>2</v>
+      </c>
+      <c r="G10" t="s">
+        <v>1009</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>157</v>
+      </c>
+      <c r="B11" t="s">
+        <v>1003</v>
+      </c>
+      <c r="C11" t="s">
+        <v>1004</v>
+      </c>
+      <c r="D11" t="s">
+        <v>234</v>
+      </c>
+      <c r="E11">
+        <v>50</v>
+      </c>
+      <c r="F11">
+        <v>1</v>
+      </c>
+      <c r="G11" t="s">
+        <v>1009</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>1012</v>
+      </c>
+      <c r="B12" t="s">
+        <v>1003</v>
+      </c>
+      <c r="C12" t="s">
+        <v>229</v>
+      </c>
+      <c r="D12" t="s">
+        <v>1004</v>
+      </c>
+      <c r="E12">
+        <v>0</v>
+      </c>
+      <c r="F12">
+        <v>1</v>
+      </c>
+      <c r="G12" t="s">
+        <v>1009</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>184</v>
+      </c>
+      <c r="B13" t="s">
+        <v>1003</v>
+      </c>
+      <c r="C13" t="s">
+        <v>1004</v>
+      </c>
+      <c r="D13" t="s">
+        <v>229</v>
+      </c>
+      <c r="E13">
+        <v>0</v>
+      </c>
+      <c r="F13">
+        <v>1</v>
+      </c>
+      <c r="G13" t="s">
+        <v>1009</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:G51" xr:uid="{00000000-0009-0000-0000-000008000000}"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0900-000000000000}">
   <dimension ref="A1:C14"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -7285,7 +7609,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0A00-000000000000}">
   <dimension ref="A1:R24"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -8660,6 +8984,349 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{86FCEC72-F57A-476F-86FC-E29836F3A0C3}">
+  <dimension ref="A1:K19"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="22.21875" customWidth="1"/>
+    <col min="3" max="3" width="16.5546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="7.6640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="5.21875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="18" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="7.6640625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="5.21875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A1" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="C1" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>997</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>1080</v>
+      </c>
+      <c r="G1" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>997</v>
+      </c>
+      <c r="I1" s="3" t="s">
+        <v>1080</v>
+      </c>
+      <c r="K1" s="5"/>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A2" s="6" t="s">
+        <v>4</v>
+      </c>
+      <c r="C2" s="8" t="s">
+        <v>596</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>1081</v>
+      </c>
+      <c r="E2" s="3">
+        <v>103</v>
+      </c>
+      <c r="G2" s="8" t="s">
+        <v>690</v>
+      </c>
+      <c r="H2" s="6" t="s">
+        <v>1081</v>
+      </c>
+      <c r="I2" s="6">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A3" s="5" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A4" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>997</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>1080</v>
+      </c>
+      <c r="G4" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="H4" s="3" t="s">
+        <v>997</v>
+      </c>
+      <c r="I4" s="3" t="s">
+        <v>1080</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A5" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="C5" s="8" t="s">
+        <v>616</v>
+      </c>
+      <c r="D5" s="6" t="s">
+        <v>1081</v>
+      </c>
+      <c r="E5" s="6">
+        <v>107</v>
+      </c>
+      <c r="G5" s="8" t="s">
+        <v>611</v>
+      </c>
+      <c r="H5" s="6" t="s">
+        <v>1081</v>
+      </c>
+      <c r="I5" s="6">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A6" s="3" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A7" s="5" t="s">
+        <v>69</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>997</v>
+      </c>
+      <c r="E7" s="3" t="s">
+        <v>1080</v>
+      </c>
+      <c r="G7" s="3" t="s">
+        <v>119</v>
+      </c>
+      <c r="H7" s="3" t="s">
+        <v>997</v>
+      </c>
+      <c r="I7" s="3" t="s">
+        <v>1080</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A8" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="C8" s="8" t="s">
+        <v>915</v>
+      </c>
+      <c r="D8" s="6" t="s">
+        <v>1081</v>
+      </c>
+      <c r="E8" s="6">
+        <v>102</v>
+      </c>
+      <c r="G8" s="3" t="s">
+        <v>698</v>
+      </c>
+      <c r="H8" s="6" t="s">
+        <v>1082</v>
+      </c>
+      <c r="I8" s="6">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A9" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="G9" s="3" t="s">
+        <v>644</v>
+      </c>
+      <c r="H9" s="6" t="s">
+        <v>1081</v>
+      </c>
+      <c r="I9" s="6">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A10" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="D10" s="3" t="s">
+        <v>997</v>
+      </c>
+      <c r="E10" s="3" t="s">
+        <v>1080</v>
+      </c>
+      <c r="G10" s="3" t="s">
+        <v>590</v>
+      </c>
+      <c r="H10" s="12" t="s">
+        <v>1082</v>
+      </c>
+      <c r="I10" s="6">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A11" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="C11" s="8" t="s">
+        <v>619</v>
+      </c>
+      <c r="D11" s="6" t="s">
+        <v>1081</v>
+      </c>
+      <c r="E11" s="6">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A12" s="3" t="s">
+        <v>119</v>
+      </c>
+      <c r="G12" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="H12" s="3" t="s">
+        <v>997</v>
+      </c>
+      <c r="I12" s="3" t="s">
+        <v>1080</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A13" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="C13" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="D13" s="3" t="s">
+        <v>997</v>
+      </c>
+      <c r="E13" s="3" t="s">
+        <v>1080</v>
+      </c>
+      <c r="G13" s="8" t="s">
+        <v>909</v>
+      </c>
+      <c r="H13" s="12" t="s">
+        <v>1081</v>
+      </c>
+      <c r="I13" s="6">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A14" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="C14" s="8" t="s">
+        <v>553</v>
+      </c>
+      <c r="D14" s="6" t="s">
+        <v>1081</v>
+      </c>
+      <c r="E14" s="6">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A15" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="C15" s="8" t="s">
+        <v>571</v>
+      </c>
+      <c r="D15" s="6" t="s">
+        <v>1082</v>
+      </c>
+      <c r="E15" s="6">
+        <v>105</v>
+      </c>
+      <c r="G15" s="3" t="s">
+        <v>193</v>
+      </c>
+      <c r="H15" s="3" t="s">
+        <v>997</v>
+      </c>
+      <c r="I15" s="3" t="s">
+        <v>1080</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A16" s="3" t="s">
+        <v>193</v>
+      </c>
+      <c r="G16" s="6" t="s">
+        <v>1083</v>
+      </c>
+      <c r="H16" s="12" t="s">
+        <v>1081</v>
+      </c>
+      <c r="I16" s="6">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A17" s="3" t="s">
+        <v>259</v>
+      </c>
+      <c r="C17" s="5" t="s">
+        <v>69</v>
+      </c>
+      <c r="D17" s="3" t="s">
+        <v>997</v>
+      </c>
+      <c r="E17" s="3" t="s">
+        <v>1080</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="C18" s="8" t="s">
+        <v>584</v>
+      </c>
+      <c r="D18" s="6" t="s">
+        <v>1081</v>
+      </c>
+      <c r="E18" s="6">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="C19" s="8" t="s">
+        <v>836</v>
+      </c>
+      <c r="D19" s="6" t="s">
+        <v>1082</v>
+      </c>
+      <c r="E19" s="6">
+        <v>105</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:F8"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -8833,7 +9500,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:F8"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -9007,7 +9674,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:D249"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -11360,7 +12027,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:D250"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -13431,7 +14098,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:R24"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -14805,7 +15472,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <dimension ref="A1:AN24"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -16179,7 +16846,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
   <dimension ref="A1:H19"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -16692,312 +17359,4 @@
   </autoFilter>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
-  <dimension ref="A1:G13"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="1" width="16.6640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="17.21875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="15.6640625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="16.44140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="5.77734375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="11.109375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="30.77734375" customWidth="1"/>
-    <col min="8" max="10" width="8.77734375" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A1" t="s">
-        <v>1</v>
-      </c>
-      <c r="B1" t="s">
-        <v>997</v>
-      </c>
-      <c r="C1" t="s">
-        <v>998</v>
-      </c>
-      <c r="D1" t="s">
-        <v>999</v>
-      </c>
-      <c r="E1" t="s">
-        <v>1000</v>
-      </c>
-      <c r="F1" t="s">
-        <v>1001</v>
-      </c>
-      <c r="G1" t="s">
-        <v>1002</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
-        <v>464</v>
-      </c>
-      <c r="B2" t="s">
-        <v>1003</v>
-      </c>
-      <c r="C2" t="s">
-        <v>229</v>
-      </c>
-      <c r="D2" t="s">
-        <v>1004</v>
-      </c>
-      <c r="F2">
-        <v>1</v>
-      </c>
-      <c r="G2" t="s">
-        <v>1005</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
-        <v>1006</v>
-      </c>
-      <c r="B3" t="s">
-        <v>1003</v>
-      </c>
-      <c r="C3" t="s">
-        <v>1004</v>
-      </c>
-      <c r="D3" t="s">
-        <v>229</v>
-      </c>
-      <c r="F3">
-        <v>1</v>
-      </c>
-      <c r="G3" t="s">
-        <v>1005</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
-        <v>57</v>
-      </c>
-      <c r="B4" t="s">
-        <v>1003</v>
-      </c>
-      <c r="C4" t="s">
-        <v>234</v>
-      </c>
-      <c r="D4" t="s">
-        <v>55</v>
-      </c>
-      <c r="F4">
-        <v>1</v>
-      </c>
-      <c r="G4" t="s">
-        <v>1005</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
-        <v>66</v>
-      </c>
-      <c r="B5" t="s">
-        <v>1003</v>
-      </c>
-      <c r="C5" t="s">
-        <v>55</v>
-      </c>
-      <c r="D5" t="s">
-        <v>234</v>
-      </c>
-      <c r="F5">
-        <v>1</v>
-      </c>
-      <c r="G5" t="s">
-        <v>1005</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
-        <v>1007</v>
-      </c>
-      <c r="B6" t="s">
-        <v>1003</v>
-      </c>
-      <c r="C6" t="s">
-        <v>501</v>
-      </c>
-      <c r="D6" t="s">
-        <v>234</v>
-      </c>
-      <c r="E6">
-        <v>40</v>
-      </c>
-      <c r="F6">
-        <v>2</v>
-      </c>
-      <c r="G6" t="s">
-        <v>1005</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
-        <v>267</v>
-      </c>
-      <c r="B7" t="s">
-        <v>1003</v>
-      </c>
-      <c r="C7" t="s">
-        <v>501</v>
-      </c>
-      <c r="D7" t="s">
-        <v>234</v>
-      </c>
-      <c r="E7">
-        <v>15</v>
-      </c>
-      <c r="F7">
-        <v>2</v>
-      </c>
-      <c r="G7" t="s">
-        <v>1005</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A8" t="s">
-        <v>1008</v>
-      </c>
-      <c r="B8" t="s">
-        <v>1003</v>
-      </c>
-      <c r="C8" t="s">
-        <v>234</v>
-      </c>
-      <c r="D8" t="s">
-        <v>497</v>
-      </c>
-      <c r="E8">
-        <v>0</v>
-      </c>
-      <c r="F8">
-        <v>2</v>
-      </c>
-      <c r="G8" t="s">
-        <v>1009</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A9" t="s">
-        <v>1010</v>
-      </c>
-      <c r="B9" t="s">
-        <v>1003</v>
-      </c>
-      <c r="C9" t="s">
-        <v>229</v>
-      </c>
-      <c r="D9" t="s">
-        <v>233</v>
-      </c>
-      <c r="E9">
-        <v>0</v>
-      </c>
-      <c r="F9">
-        <v>2</v>
-      </c>
-      <c r="G9" t="s">
-        <v>1009</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A10" t="s">
-        <v>1011</v>
-      </c>
-      <c r="B10" t="s">
-        <v>1003</v>
-      </c>
-      <c r="C10" t="s">
-        <v>233</v>
-      </c>
-      <c r="D10" t="s">
-        <v>229</v>
-      </c>
-      <c r="E10">
-        <v>0</v>
-      </c>
-      <c r="F10">
-        <v>2</v>
-      </c>
-      <c r="G10" t="s">
-        <v>1009</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A11" t="s">
-        <v>157</v>
-      </c>
-      <c r="B11" t="s">
-        <v>1003</v>
-      </c>
-      <c r="C11" t="s">
-        <v>1004</v>
-      </c>
-      <c r="D11" t="s">
-        <v>234</v>
-      </c>
-      <c r="E11">
-        <v>50</v>
-      </c>
-      <c r="F11">
-        <v>1</v>
-      </c>
-      <c r="G11" t="s">
-        <v>1009</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A12" t="s">
-        <v>1012</v>
-      </c>
-      <c r="B12" t="s">
-        <v>1003</v>
-      </c>
-      <c r="C12" t="s">
-        <v>229</v>
-      </c>
-      <c r="D12" t="s">
-        <v>1004</v>
-      </c>
-      <c r="E12">
-        <v>0</v>
-      </c>
-      <c r="F12">
-        <v>1</v>
-      </c>
-      <c r="G12" t="s">
-        <v>1009</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A13" t="s">
-        <v>184</v>
-      </c>
-      <c r="B13" t="s">
-        <v>1003</v>
-      </c>
-      <c r="C13" t="s">
-        <v>1004</v>
-      </c>
-      <c r="D13" t="s">
-        <v>229</v>
-      </c>
-      <c r="E13">
-        <v>0</v>
-      </c>
-      <c r="F13">
-        <v>1</v>
-      </c>
-      <c r="G13" t="s">
-        <v>1009</v>
-      </c>
-    </row>
-  </sheetData>
-  <autoFilter ref="A1:G51" xr:uid="{00000000-0009-0000-0000-000008000000}"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Actualización automática de base de datos y web
</commit_message>
<xml_diff>
--- a/LMI Base.xlsx
+++ b/LMI Base.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\alex1\Downloads\LMI\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D61601FE-001E-4874-AA52-8337C6468984}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{32ACBB55-DAF9-4EF0-9387-56A43F50118F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="4" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Registro Liga" sheetId="1" r:id="rId1"/>
@@ -3429,7 +3429,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -3458,9 +3458,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -9176,7 +9173,7 @@
       <c r="G10" s="3" t="s">
         <v>590</v>
       </c>
-      <c r="H10" s="12" t="s">
+      <c r="H10" s="3" t="s">
         <v>1082</v>
       </c>
       <c r="I10" s="6">
@@ -9227,7 +9224,7 @@
       <c r="G13" s="8" t="s">
         <v>909</v>
       </c>
-      <c r="H13" s="12" t="s">
+      <c r="H13" s="3" t="s">
         <v>1081</v>
       </c>
       <c r="I13" s="6">
@@ -9278,7 +9275,7 @@
       <c r="G16" s="6" t="s">
         <v>1083</v>
       </c>
-      <c r="H16" s="12" t="s">
+      <c r="H16" s="3" t="s">
         <v>1081</v>
       </c>
       <c r="I16" s="6">
@@ -16955,7 +16952,7 @@
         <v>100000000</v>
       </c>
       <c r="F4" s="7">
-        <v>8100000000</v>
+        <v>810000000</v>
       </c>
       <c r="G4" t="s">
         <v>937</v>

</xml_diff>

<commit_message>
Actualizar base de datos con nuevo club (River Plate) y habilitar despliegue directo a producción en gestor de clubes
</commit_message>
<xml_diff>
--- a/LMI Base.xlsx
+++ b/LMI Base.xlsx
@@ -581,7 +581,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E247"/>
+  <dimension ref="A1:D247"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4"/>
   <cols>
     <col width="16.88671875" bestFit="1" customWidth="1" style="1" min="1" max="1"/>
@@ -13790,7 +13790,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q24"/>
+  <dimension ref="A1:R24"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4"/>
   <cols>
     <col width="17.77734375" bestFit="1" customWidth="1" style="4" min="1" max="1"/>
@@ -13899,6 +13899,11 @@
           <t>Club_America</t>
         </is>
       </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>Club_Atlético_River_Plate</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
@@ -13986,6 +13991,11 @@
           <t>Yann Sommer</t>
         </is>
       </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>Orlando Gill</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
@@ -14073,6 +14083,11 @@
           <t>Luke Shaw</t>
         </is>
       </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>Maarten Paes</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
@@ -14160,6 +14175,11 @@
           <t>Alessandro Deiola</t>
         </is>
       </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>Trevoh Chalobah</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
@@ -14247,6 +14267,11 @@
           <t>Amir Rrahmani</t>
         </is>
       </c>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>Manuel Akanji</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
@@ -14334,6 +14359,11 @@
           <t>Joshua Kimmich</t>
         </is>
       </c>
+      <c r="R6" t="inlineStr">
+        <is>
+          <t>Strahinja Pavlović</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
@@ -14421,6 +14451,11 @@
           <t>Sergio Busquets</t>
         </is>
       </c>
+      <c r="R7" t="inlineStr">
+        <is>
+          <t>Jérémy Jacquet</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
@@ -14508,6 +14543,11 @@
           <t>Seko Fofana</t>
         </is>
       </c>
+      <c r="R8" t="inlineStr">
+        <is>
+          <t>Raphaël Guerreiro</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
@@ -14595,6 +14635,11 @@
           <t>Lee Jae-sung</t>
         </is>
       </c>
+      <c r="R9" t="inlineStr">
+        <is>
+          <t>Ainsley Maitland-Niles</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
@@ -14682,6 +14727,11 @@
           <t>Rodrigo Garro</t>
         </is>
       </c>
+      <c r="R10" t="inlineStr">
+        <is>
+          <t>Gonzalo Montiel</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
@@ -14769,6 +14819,11 @@
           <t>Gerard Moreno</t>
         </is>
       </c>
+      <c r="R11" t="inlineStr">
+        <is>
+          <t>Danilo</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
@@ -14856,6 +14911,11 @@
           <t>Alessandro Del Piero</t>
         </is>
       </c>
+      <c r="R12" t="inlineStr">
+        <is>
+          <t>D Máximo Perrone</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
@@ -14943,6 +15003,11 @@
           <t>Lucas Perri</t>
         </is>
       </c>
+      <c r="R13" t="inlineStr">
+        <is>
+          <t>D Johnny Cardoso</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
@@ -15030,6 +15095,11 @@
           <t>Sebastián Cáceres</t>
         </is>
       </c>
+      <c r="R14" t="inlineStr">
+        <is>
+          <t>Thiago Pitarch</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
@@ -15117,6 +15187,11 @@
           <t>Miguel Layún</t>
         </is>
       </c>
+      <c r="R15" t="inlineStr">
+        <is>
+          <t>Valentín Barco</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
@@ -15204,6 +15279,11 @@
           <t>Lucas Digne</t>
         </is>
       </c>
+      <c r="R16" t="inlineStr">
+        <is>
+          <t>ID Bernardo Silva</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
@@ -15291,6 +15371,11 @@
           <t>Ross Barkley</t>
         </is>
       </c>
+      <c r="R17" t="inlineStr">
+        <is>
+          <t>II Emam Ashour</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
@@ -15378,6 +15463,11 @@
           <t>Yacine Adli</t>
         </is>
       </c>
+      <c r="R18" t="inlineStr">
+        <is>
+          <t>II Exequiel Zeballos</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="5" t="inlineStr">
@@ -15465,6 +15555,11 @@
           <t>Álvaro Fidalgo</t>
         </is>
       </c>
+      <c r="R19" t="inlineStr">
+        <is>
+          <t>Alan Patrick</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="5" t="inlineStr">
@@ -15552,6 +15647,11 @@
           <t>Tommaso Baldanzi</t>
         </is>
       </c>
+      <c r="R20" t="inlineStr">
+        <is>
+          <t>Ibrahim Mbaye</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="5" t="inlineStr">
@@ -15639,6 +15739,11 @@
           <t>Olivier Giroud</t>
         </is>
       </c>
+      <c r="R21" t="inlineStr">
+        <is>
+          <t>Moussa Diaby</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
@@ -15726,6 +15831,11 @@
           <t>Florian Thauvin</t>
         </is>
       </c>
+      <c r="R22" t="inlineStr">
+        <is>
+          <t>Pierre-Emerick Aubameyang</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="5" t="inlineStr">
@@ -15813,6 +15923,11 @@
           <t>Ciro Immobile</t>
         </is>
       </c>
+      <c r="R23" t="inlineStr">
+        <is>
+          <t>Alexander Sørloth</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
@@ -15898,6 +16013,11 @@
       <c r="Q24" s="3" t="inlineStr">
         <is>
           <t>Gabriel Barbosa</t>
+        </is>
+      </c>
+      <c r="R24" t="inlineStr">
+        <is>
+          <t>Zlatan Ibrahimović</t>
         </is>
       </c>
     </row>
@@ -15912,7 +16032,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q24"/>
+  <dimension ref="A1:R24"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4"/>
   <cols>
     <col width="23.44140625" bestFit="1" customWidth="1" style="11" min="1" max="1"/>
@@ -16021,6 +16141,11 @@
           <t>Club America</t>
         </is>
       </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>Club Atlético River Plate</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="8" t="inlineStr">
@@ -16108,6 +16233,11 @@
           <t>PT Yann Sommer</t>
         </is>
       </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>PT Orlando Gill</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="8" t="inlineStr">
@@ -16195,6 +16325,11 @@
           <t>LI Luke Shaw</t>
         </is>
       </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>PT Maarten Paes</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="8" t="inlineStr">
@@ -16282,6 +16417,11 @@
           <t>MC Alessandro Deiola</t>
         </is>
       </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>CT Trevoh Chalobah</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="8" t="inlineStr">
@@ -16369,6 +16509,11 @@
           <t>CT Amir Rrahmani</t>
         </is>
       </c>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>CT Manuel Akanji</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="8" t="inlineStr">
@@ -16456,6 +16601,11 @@
           <t>MCD Joshua Kimmich</t>
         </is>
       </c>
+      <c r="R6" t="inlineStr">
+        <is>
+          <t>CT Strahinja Pavlović</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="8" t="inlineStr">
@@ -16543,6 +16693,11 @@
           <t>MCD Sergio Busquets</t>
         </is>
       </c>
+      <c r="R7" t="inlineStr">
+        <is>
+          <t>CT Jérémy Jacquet</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="8" t="inlineStr">
@@ -16630,6 +16785,11 @@
           <t>MC Seko Fofana</t>
         </is>
       </c>
+      <c r="R8" t="inlineStr">
+        <is>
+          <t>LI Raphaël Guerreiro</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="8" t="inlineStr">
@@ -16717,6 +16877,11 @@
           <t>MP Lee Jae-sung</t>
         </is>
       </c>
+      <c r="R9" t="inlineStr">
+        <is>
+          <t>LD Ainsley Maitland-Niles</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="8" t="inlineStr">
@@ -16804,6 +16969,11 @@
           <t>MP Rodrigo Garro</t>
         </is>
       </c>
+      <c r="R10" t="inlineStr">
+        <is>
+          <t>LD Gonzalo Montiel</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="8" t="inlineStr">
@@ -16891,6 +17061,11 @@
           <t>DC Gerard Moreno</t>
         </is>
       </c>
+      <c r="R11" t="inlineStr">
+        <is>
+          <t>LD Danilo</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="8" t="inlineStr">
@@ -16978,6 +17153,11 @@
           <t>DC Alessandro Del Piero</t>
         </is>
       </c>
+      <c r="R12" t="inlineStr">
+        <is>
+          <t>MCD Máximo Perrone</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="8" t="inlineStr">
@@ -17065,6 +17245,11 @@
           <t>PT Lucas Perri</t>
         </is>
       </c>
+      <c r="R13" t="inlineStr">
+        <is>
+          <t>MCD Johnny Cardoso</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="8" t="inlineStr">
@@ -17152,6 +17337,11 @@
           <t>CT Sebastián Cáceres</t>
         </is>
       </c>
+      <c r="R14" t="inlineStr">
+        <is>
+          <t>MC Thiago Pitarch</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="8" t="inlineStr">
@@ -17239,6 +17429,11 @@
           <t>LD Miguel Layún</t>
         </is>
       </c>
+      <c r="R15" t="inlineStr">
+        <is>
+          <t>MC Valentín Barco</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="8" t="inlineStr">
@@ -17326,6 +17521,11 @@
           <t>LI Lucas Digne</t>
         </is>
       </c>
+      <c r="R16" t="inlineStr">
+        <is>
+          <t>ID Bernardo Silva</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="8" t="inlineStr">
@@ -17413,6 +17613,11 @@
           <t>MC Ross Barkley</t>
         </is>
       </c>
+      <c r="R17" t="inlineStr">
+        <is>
+          <t>II Emam Ashour</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="8" t="inlineStr">
@@ -17500,6 +17705,11 @@
           <t>MC Yacine Adli</t>
         </is>
       </c>
+      <c r="R18" t="inlineStr">
+        <is>
+          <t>II Exequiel Zeballos</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="8" t="inlineStr">
@@ -17587,6 +17797,11 @@
           <t>MC Álvaro Fidalgo</t>
         </is>
       </c>
+      <c r="R19" t="inlineStr">
+        <is>
+          <t>MP Alan Patrick</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="8" t="inlineStr">
@@ -17674,6 +17889,11 @@
           <t>MP Tommaso Baldanzi</t>
         </is>
       </c>
+      <c r="R20" t="inlineStr">
+        <is>
+          <t>ED Ibrahim Mbaye</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="8" t="inlineStr">
@@ -17761,6 +17981,11 @@
           <t>DC Olivier Giroud</t>
         </is>
       </c>
+      <c r="R21" t="inlineStr">
+        <is>
+          <t>ED Moussa Diaby</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="8" t="inlineStr">
@@ -17848,6 +18073,11 @@
           <t>ED Florian Thauvin</t>
         </is>
       </c>
+      <c r="R22" t="inlineStr">
+        <is>
+          <t>DC Pierre-Emerick Aubameyang</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="8" t="inlineStr">
@@ -17935,6 +18165,11 @@
           <t>DC Ciro Immobile</t>
         </is>
       </c>
+      <c r="R23" t="inlineStr">
+        <is>
+          <t>DC Alexander Sørloth</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="8" t="inlineStr">
@@ -18020,6 +18255,11 @@
       <c r="Q24" s="8" t="inlineStr">
         <is>
           <t>DC Gabriel Barbosa</t>
+        </is>
+      </c>
+      <c r="R24" t="inlineStr">
+        <is>
+          <t>DC Zlatan Ibrahimović</t>
         </is>
       </c>
     </row>
@@ -18034,7 +18274,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H18"/>
+  <dimension ref="A1:H19"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
   <cols>
     <col width="18.88671875" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -18734,6 +18974,48 @@
         </is>
       </c>
     </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Club Atlético River Plate</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>RVP</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Estadio Monumental</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Parraga</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>300000000</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>300000000</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>Logos Equipos/riverplate.webp</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:H19">
     <sortState ref="A2:H19">

</xml_diff>